<commit_message>
Document CRC microbiome pilot analysis
</commit_message>
<xml_diff>
--- a/results/alpha-diversity-all-metrics.xlsx
+++ b/results/alpha-diversity-all-metrics.xlsx
@@ -7,9 +7,13 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rarefied (15000)" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Rarefied (15000)'!$A$1:$E$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Notes'!$A$1:$A$5</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -17,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,13 +32,22 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00274C77"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -55,10 +68,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -427,29 +443,36 @@
   </sheetPr>
   <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Sample ID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Group</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>Shannon</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Simpson</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Simpson (QIIME 2 metric)</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>Pielou evenness</t>
         </is>
@@ -463,17 +486,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>normal</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>4.631383310556756</v>
+        <v>4.646449150952917</v>
       </c>
       <c r="D2" t="n">
-        <v>0.9173251007479722</v>
+        <v>0.9186154933333334</v>
       </c>
       <c r="E2" t="n">
-        <v>0.6671045925788019</v>
+        <v>0.6812796521262396</v>
       </c>
     </row>
     <row r="3">
@@ -484,17 +507,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>cancer</t>
+          <t>Cancer</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>5.155210210462991</v>
+        <v>5.148121732840227</v>
       </c>
       <c r="D3" t="n">
-        <v>0.9466484206018972</v>
+        <v>0.9471658222222222</v>
       </c>
       <c r="E3" t="n">
-        <v>0.7023590684328629</v>
+        <v>0.7075362440351505</v>
       </c>
     </row>
     <row r="4">
@@ -505,17 +528,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>normal</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>5.56768242803812</v>
+        <v>5.568746284351269</v>
       </c>
       <c r="D4" t="n">
-        <v>0.9551909573495618</v>
+        <v>0.9554836177777778</v>
       </c>
       <c r="E4" t="n">
-        <v>0.7385018100208763</v>
+        <v>0.740174177720172</v>
       </c>
     </row>
     <row r="5">
@@ -526,17 +549,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>cancer</t>
+          <t>Cancer</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>4.68600696934316</v>
+        <v>4.682999858791417</v>
       </c>
       <c r="D5" t="n">
-        <v>0.8765036140876949</v>
+        <v>0.8759765511111111</v>
       </c>
       <c r="E5" t="n">
-        <v>0.6159857369245024</v>
+        <v>0.6198881171079839</v>
       </c>
     </row>
     <row r="6">
@@ -547,17 +570,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>normal</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>5.982980002374452</v>
+        <v>5.970706542024882</v>
       </c>
       <c r="D6" t="n">
-        <v>0.9709272259416428</v>
+        <v>0.97103048</v>
       </c>
       <c r="E6" t="n">
-        <v>0.7468244017574502</v>
+        <v>0.7592275198220606</v>
       </c>
     </row>
     <row r="7">
@@ -568,17 +591,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>adenoma</t>
+          <t>Adenoma</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>5.654421256446641</v>
+        <v>5.653238399490938</v>
       </c>
       <c r="D7" t="n">
-        <v>0.9663969739021744</v>
+        <v>0.9664952711111111</v>
       </c>
       <c r="E7" t="n">
-        <v>0.8245023222525653</v>
+        <v>0.824329843361687</v>
       </c>
     </row>
     <row r="8">
@@ -589,17 +612,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>adenoma</t>
+          <t>Adenoma</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>4.858351770155323</v>
+        <v>4.82741277113568</v>
       </c>
       <c r="D8" t="n">
-        <v>0.9273480608470458</v>
+        <v>0.9259581333333333</v>
       </c>
       <c r="E8" t="n">
-        <v>0.7046381698454666</v>
+        <v>0.7001508867755222</v>
       </c>
     </row>
     <row r="9">
@@ -610,17 +633,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>cancer</t>
+          <t>Cancer</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>6.108376562066769</v>
+        <v>6.090140324309522</v>
       </c>
       <c r="D9" t="n">
-        <v>0.9657936926339176</v>
+        <v>0.9658485511111111</v>
       </c>
       <c r="E9" t="n">
-        <v>0.7344082644111866</v>
+        <v>0.743622806633402</v>
       </c>
     </row>
     <row r="10">
@@ -631,20 +654,74 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>adenoma</t>
+          <t>Adenoma</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>5.808992043487754</v>
+        <v>5.789835239773351</v>
       </c>
       <c r="D10" t="n">
-        <v>0.972136988091919</v>
+        <v>0.9719580355555556</v>
       </c>
       <c r="E10" t="n">
-        <v>0.7885878291141918</v>
+        <v>0.7897832339441823</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:E10"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="90" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Alpha-diversity metrics calculated from the QIIME 2 feature table rarefied to 15,000 reads per sample.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Groups are taken from the dx column in qiime-metadata.tsv.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>The Simpson column contains values returned by QIIME 2's simpson metric; retain this label rather than inferring direction from an internal function name.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>There are 3 samples per group; treat group comparisons as exploratory.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:A5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>